<commit_message>
add generic growth rates; placeholder SD for Porites mortality
</commit_message>
<xml_diff>
--- a/www/Baseline_Cover_TEMPLATE.xlsx
+++ b/www/Baseline_Cover_TEMPLATE.xlsx
@@ -8,22 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\__git\CBuRT\www\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{936F06E3-E98A-4A5C-A5E4-FDCC7E695BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC659CD8-54D9-46A4-BE1A-EF15853E462A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3953" yWindow="3953" windowWidth="21599" windowHeight="11332" activeTab="1" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
+    <workbookView xWindow="3128" yWindow="3128" windowWidth="21600" windowHeight="11332" activeTab="2" xr2:uid="{0278FB9D-D97A-43A8-AA68-A0B70EFAF30B}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="3" r:id="rId1"/>
     <sheet name="Coral Cover input" sheetId="1" r:id="rId2"/>
     <sheet name="Taxa" sheetId="2" r:id="rId3"/>
-    <sheet name="Metadata" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="RangeA">Metadata!$B$2:$B$4</definedName>
-    <definedName name="RangeDRTO">Metadata!$B$5:$B$7</definedName>
-    <definedName name="SEFCRI">Metadata!$B$8</definedName>
-    <definedName name="SubregionList">Metadata!$A$2:$A$5</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -48,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="88">
   <si>
     <t>Acropora cervicornis</t>
   </si>
@@ -77,9 +70,6 @@
     <t>Agaricia tenuifolia</t>
   </si>
   <si>
-    <t>Agaricia undata</t>
-  </si>
-  <si>
     <t>Crustose coralline algae</t>
   </si>
   <si>
@@ -215,27 +205,15 @@
     <t>Stephanocoenia intersepta</t>
   </si>
   <si>
-    <t>Stylaster roseus</t>
-  </si>
-  <si>
     <t>Tubastraea coccinea</t>
   </si>
   <si>
     <t>Taxon</t>
   </si>
   <si>
-    <t>Acropora spp.</t>
-  </si>
-  <si>
     <t>Agaricia spp.</t>
   </si>
   <si>
-    <t>Favia spp.</t>
-  </si>
-  <si>
-    <t>Isophyllia spp.</t>
-  </si>
-  <si>
     <t>Madracis spp.</t>
   </si>
   <si>
@@ -245,25 +223,10 @@
     <t>Mycetophyllia spp.</t>
   </si>
   <si>
-    <t>Oculina spp.</t>
-  </si>
-  <si>
     <t>Orbicella spp.</t>
   </si>
   <si>
-    <t>Porites spp.</t>
-  </si>
-  <si>
     <t>Pseudodiploria spp.</t>
-  </si>
-  <si>
-    <t>Siderastrea spp.</t>
-  </si>
-  <si>
-    <t>Scolymia spp.</t>
-  </si>
-  <si>
-    <t>Solenastrea spp.</t>
   </si>
   <si>
     <t>Site_Name</t>
@@ -389,51 +352,6 @@
   </si>
   <si>
     <t>•  Please provide a point of contact (POC) first and last name and email for the baseline site data so that we can contact you with questions, if necessary</t>
-  </si>
-  <si>
-    <t>Habitat_FK</t>
-  </si>
-  <si>
-    <t>DryTortugas</t>
-  </si>
-  <si>
-    <t>Inshore</t>
-  </si>
-  <si>
-    <t>LowerKeys</t>
-  </si>
-  <si>
-    <t>MidChannel</t>
-  </si>
-  <si>
-    <t>MiddleKeys</t>
-  </si>
-  <si>
-    <t>Offshore</t>
-  </si>
-  <si>
-    <t>UpperKeys</t>
-  </si>
-  <si>
-    <t>Bank</t>
-  </si>
-  <si>
-    <t>Biscayne</t>
-  </si>
-  <si>
-    <t>Lagoon</t>
-  </si>
-  <si>
-    <t>SoutheastFlorida</t>
-  </si>
-  <si>
-    <t>ForeReef</t>
-  </si>
-  <si>
-    <t>SEFCRI</t>
-  </si>
-  <si>
-    <t>Tubastraea spp.</t>
   </si>
   <si>
     <t>REQUIRED Unconsolidated substrate</t>
@@ -863,22 +781,22 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -886,47 +804,47 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>92</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>96</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -939,59 +857,59 @@
   <dimension ref="A1:K1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="5.796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.46484375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.265625" customWidth="1"/>
+    <col min="2" max="2" width="12.3984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9.1328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.86328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.1328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.53125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.59765625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.3984375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.86328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.06640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="9.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B1" t="s">
-        <v>79</v>
+        <v>69</v>
       </c>
       <c r="C1" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="D1" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="F1" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="G1" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="H1" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="I1" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="J1" t="s">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="K1" t="s">
-        <v>95</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{268EBEEC-525C-485A-BCB7-2F826408B174}">
-      <formula1>IF(C2="DryTortugas",        RangeDRTO,    IF(ISNUMBER(MATCH(C2, SubregionList, 0)),        RangeA,     SEFCRI))</formula1>
+      <formula1>"Inshore, MidChannel, Offshore, Bank, Lagoon, ForeReef"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{2551E9F4-EAD3-4C0C-A0CF-00F9C4CBBDD7}">
       <formula1>"DryTortugas, LowerKeys,MiddleKeys, UpperKeys, Biscayne, SoutheastFlorida"</formula1>
@@ -1003,9 +921,9 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{101649E4-CD8D-4DAA-89FC-8D6C93B48E30}">
           <x14:formula1>
-            <xm:f>Taxa!$A$2:$A$76</xm:f>
+            <xm:f>Taxa!$A$2:$A$65</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A1048576</xm:sqref>
+          <xm:sqref>A3:A1048576 A2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1015,77 +933,77 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAEEECA6-441C-430E-B4E3-69F7F23BD6EB}">
-  <dimension ref="A1:A76"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>59</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>9</v>
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.45">
@@ -1095,395 +1013,261 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>61</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A32" t="s">
-        <v>23</v>
+      <c r="A32" s="1" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A36" s="1" t="s">
-        <v>63</v>
+      <c r="A36" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>33</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>81</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>40</v>
+        <v>61</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>68</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>53</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A66" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A67" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A68" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A69" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A70" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A71" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A72" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A73" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A74" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A75" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A76" t="s">
-        <v>56</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58E31873-3B71-4C96-9888-7DA8F3D3EA70}">
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>104</v>
-      </c>
-      <c r="B4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="B8" t="s">
-        <v>110</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="797e7fd4-719a-42b3-b312-968ffa9058ad">
@@ -1494,9 +1278,9 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ca57789ecb406bb7a99068f68ac4c0ed">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="89dc4794f4784a0bac47690674a3da53" ns2:_="" ns3:_="">
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101000AA90A7536739341825FB392424435FB" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="647735499ae6baa62e6fc7f5ed3567b4">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="797e7fd4-719a-42b3-b312-968ffa9058ad" xmlns:ns3="811eef35-9bdd-441e-81aa-50455f68c6c3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="47ff4a2bf1fedf465812d90a21a07c12" ns2:_="" ns3:_="">
     <xsd:import namespace="797e7fd4-719a-42b3-b312-968ffa9058ad"/>
     <xsd:import namespace="811eef35-9bdd-441e-81aa-50455f68c6c3"/>
     <xsd:element name="properties">
@@ -1689,15 +1473,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9D3406C-31AD-4E38-96F6-B0246BC4EAE6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1708,8 +1493,8 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D5B4E66-2F53-40AB-B6DF-59838CE46951}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28BE2C18-A8FE-44F8-9370-C2AF79093B54}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -1727,6 +1512,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D6BB395-747F-41BC-A23A-168993E4FE92}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{6dd02d64-b7f3-43f7-a145-cfd68d338edf}" enabled="1" method="Standard" siteId="{0693b5ba-4b18-4d7b-9341-f32f400a5494}" removed="0"/>

</xml_diff>